<commit_message>
feat: add comprehensive GitHub Actions CI pipeline and enterprise load/security test modules with Excel report generation
</commit_message>
<xml_diff>
--- a/downloadable-artifacts/all-test-excel-reports/LoadTest_Report.xlsx
+++ b/downloadable-artifacts/all-test-excel-reports/LoadTest_Report.xlsx
@@ -4,59 +4,235 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Load Test Results" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Executive Load Summary" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Endpoint Breakdown" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Time-Series Progression" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
-  <si>
-    <t>Target URL</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="71">
+  <si>
+    <t>TURFINGTON BASELINE LOAD TEST BENCHMARK REPORT (100 VUs / 1 MIN)</t>
+  </si>
+  <si>
+    <t>Load Test Configuration</t>
+  </si>
+  <si>
+    <t>100 Virtual Users running continuously for 60 seconds</t>
+  </si>
+  <si>
+    <t>Target API Base URL</t>
+  </si>
+  <si>
+    <t>http://localhost:5000</t>
+  </si>
+  <si>
+    <t>Total Requests Executed</t>
+  </si>
+  <si>
+    <t>Throughput (Requests Per Second)</t>
+  </si>
+  <si>
+    <t>3944.24 req/sec</t>
+  </si>
+  <si>
+    <t>Average Response Time</t>
+  </si>
+  <si>
+    <t>13.59ms</t>
+  </si>
+  <si>
+    <t>Minimum Response Time (Fastest)</t>
+  </si>
+  <si>
+    <t>6ms</t>
+  </si>
+  <si>
+    <t>Maximum Response Time (Slowest)</t>
+  </si>
+  <si>
+    <t>98ms</t>
+  </si>
+  <si>
+    <t>Median Latency (P50)</t>
+  </si>
+  <si>
+    <t>12ms</t>
+  </si>
+  <si>
+    <t>90th Percentile Latency (P90)</t>
+  </si>
+  <si>
+    <t>19ms</t>
+  </si>
+  <si>
+    <t>95th Percentile Latency (P95)</t>
+  </si>
+  <si>
+    <t>22ms</t>
+  </si>
+  <si>
+    <t>99th Percentile Latency (P99)</t>
+  </si>
+  <si>
+    <t>29ms</t>
+  </si>
+  <si>
+    <t>Successful Requests (2xx/3xx)</t>
+  </si>
+  <si>
+    <t>Failed Requests (4xx/5xx/Timeout)</t>
+  </si>
+  <si>
+    <t>Overall Success SLA Rate</t>
+  </si>
+  <si>
+    <t>100.00%</t>
+  </si>
+  <si>
+    <t>Endpoint Name</t>
+  </si>
+  <si>
+    <t>HTTP Path</t>
   </si>
   <si>
     <t>Total Requests</t>
   </si>
   <si>
-    <t>Concurrency</t>
-  </si>
-  <si>
-    <t>Passed Requests</t>
-  </si>
-  <si>
-    <t>Failed Requests</t>
-  </si>
-  <si>
-    <t>RPS (Throughput)</t>
-  </si>
-  <si>
-    <t>Avg Latency</t>
-  </si>
-  <si>
-    <t>P95 Latency</t>
-  </si>
-  <si>
-    <t>Pass Rate</t>
-  </si>
-  <si>
-    <t>http://localhost:5000</t>
-  </si>
-  <si>
-    <t>1657.46 req/sec</t>
-  </si>
-  <si>
-    <t>0 ms</t>
-  </si>
-  <si>
-    <t>0.00%</t>
+    <t>Throughput (RPS)</t>
+  </si>
+  <si>
+    <t>Avg Response Time</t>
+  </si>
+  <si>
+    <t>Min Response Time</t>
+  </si>
+  <si>
+    <t>Max Response Time</t>
+  </si>
+  <si>
+    <t>Success Count</t>
+  </si>
+  <si>
+    <t>Failed Count</t>
+  </si>
+  <si>
+    <t>Health Check</t>
+  </si>
+  <si>
+    <t>/api/health</t>
+  </si>
+  <si>
+    <t>788.86 req/sec</t>
+  </si>
+  <si>
+    <t>13.51ms</t>
+  </si>
+  <si>
+    <t>7ms</t>
+  </si>
+  <si>
+    <t>Venues Discovery</t>
+  </si>
+  <si>
+    <t>/api/venues</t>
+  </si>
+  <si>
+    <t>13.67ms</t>
+  </si>
+  <si>
+    <t>84ms</t>
+  </si>
+  <si>
+    <t>Community Feed Posts</t>
+  </si>
+  <si>
+    <t>/api/posts</t>
+  </si>
+  <si>
+    <t>788.84 req/sec</t>
+  </si>
+  <si>
+    <t>13.66ms</t>
+  </si>
+  <si>
+    <t>83ms</t>
+  </si>
+  <si>
+    <t>Community Groups</t>
+  </si>
+  <si>
+    <t>/api/community-groups</t>
+  </si>
+  <si>
+    <t>Payment Gateway Config</t>
+  </si>
+  <si>
+    <t>/api/payments/config</t>
+  </si>
+  <si>
+    <t>788.83 req/sec</t>
+  </si>
+  <si>
+    <t>13.54ms</t>
+  </si>
+  <si>
+    <t>Time Interval Window</t>
+  </si>
+  <si>
+    <t>Requests in Window</t>
+  </si>
+  <si>
+    <t>Window Throughput (RPS)</t>
+  </si>
+  <si>
+    <t>Avg Latency (ms)</t>
+  </si>
+  <si>
+    <t>0s - 5.0s</t>
+  </si>
+  <si>
+    <t>5s - 10.0s</t>
+  </si>
+  <si>
+    <t>10s - 15.0s</t>
+  </si>
+  <si>
+    <t>15s - 20.0s</t>
+  </si>
+  <si>
+    <t>20s - 25.0s</t>
+  </si>
+  <si>
+    <t>25s - 30.0s</t>
+  </si>
+  <si>
+    <t>30s - 35.0s</t>
+  </si>
+  <si>
+    <t>35s - 40.0s</t>
+  </si>
+  <si>
+    <t>40s - 45.0s</t>
+  </si>
+  <si>
+    <t>45s - 50.0s</t>
+  </si>
+  <si>
+    <t>50s - 55.0s</t>
+  </si>
+  <si>
+    <t>55s - 60.0s</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -66,10 +242,33 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="14"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF334155"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FF0F172A"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0F766E"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -78,11 +277,21 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="C65911"/>
+        <fgColor rgb="FF0D9488"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E293B"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -90,13 +299,51 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFE2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -436,74 +683,591 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I2"/>
+  <dimension ref="B2:F18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="35" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="1" max="1" width="4" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="6" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="C6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="C7" s="4">
+        <v>236702</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="C8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B9" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="C9" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B13" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" s="3">
+        <v>236702</v>
+      </c>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" s="3">
+        <v>0</v>
+      </c>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="B2:F3"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="C7:F7"/>
+    <mergeCell ref="C8:F8"/>
+    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="C11:F11"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="C13:F13"/>
+    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="C15:F15"/>
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="C17:F17"/>
+    <mergeCell ref="C18:F18"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="7" width="20" customWidth="1"/>
+    <col min="8" max="9" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="6">
+        <v>47341</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="6">
+        <v>47341</v>
+      </c>
+      <c r="I2" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="6">
+        <v>47341</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H3" s="6">
+        <v>47341</v>
+      </c>
+      <c r="I3" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="6">
+        <v>47340</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="H4" s="6">
+        <v>47340</v>
+      </c>
+      <c r="I4" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="6">
+        <v>47341</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B2">
-        <v>300</v>
-      </c>
-      <c r="C2">
-        <v>50</v>
-      </c>
-      <c r="D2">
+      <c r="F5" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="H5" s="6">
+        <v>47341</v>
+      </c>
+      <c r="I5" s="6">
         <v>0</v>
       </c>
-      <c r="E2">
-        <v>300</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" t="s">
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" s="6">
+        <v>47339</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="H2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I2" t="s">
-        <v>12</v>
+      <c r="G6" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="H6" s="6">
+        <v>47339</v>
+      </c>
+      <c r="I6" s="6">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" s="6">
+        <v>16090</v>
+      </c>
+      <c r="C2" s="6">
+        <v>3218</v>
+      </c>
+      <c r="D2" s="6">
+        <v>16.8</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" s="6">
+        <v>18449</v>
+      </c>
+      <c r="C3" s="6">
+        <v>3689.8</v>
+      </c>
+      <c r="D3" s="6">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="6">
+        <v>18021</v>
+      </c>
+      <c r="C4" s="6">
+        <v>3604.2</v>
+      </c>
+      <c r="D4" s="6">
+        <v>14.9</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="6">
+        <v>20329</v>
+      </c>
+      <c r="C5" s="6">
+        <v>4065.8</v>
+      </c>
+      <c r="D5" s="6">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="6">
+        <v>20628</v>
+      </c>
+      <c r="C6" s="6">
+        <v>4125.6</v>
+      </c>
+      <c r="D6" s="6">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" s="6">
+        <v>20972</v>
+      </c>
+      <c r="C7" s="6">
+        <v>4194.4</v>
+      </c>
+      <c r="D7" s="6">
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" s="6">
+        <v>19982</v>
+      </c>
+      <c r="C8" s="6">
+        <v>3996.4</v>
+      </c>
+      <c r="D8" s="6">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B9" s="6">
+        <v>20579</v>
+      </c>
+      <c r="C9" s="6">
+        <v>4115.8</v>
+      </c>
+      <c r="D9" s="6">
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B10" s="6">
+        <v>20716</v>
+      </c>
+      <c r="C10" s="6">
+        <v>4143.2</v>
+      </c>
+      <c r="D10" s="6">
+        <v>12.9</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B11" s="6">
+        <v>20778</v>
+      </c>
+      <c r="C11" s="6">
+        <v>4155.6</v>
+      </c>
+      <c r="D11" s="6">
+        <v>12.9</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B12" s="6">
+        <v>20385</v>
+      </c>
+      <c r="C12" s="6">
+        <v>4077</v>
+      </c>
+      <c r="D12" s="6">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" s="6">
+        <v>20750</v>
+      </c>
+      <c r="C13" s="6">
+        <v>4150</v>
+      </c>
+      <c r="D13" s="6">
+        <v>12.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>